<commit_message>
update ui and requirements
</commit_message>
<xml_diff>
--- a/reports/employee_safety.xlsx
+++ b/reports/employee_safety.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-02-28 15:49:51</t>
+          <t>2026-03-03 20:15:57</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-03-01 20:26:11</t>
+          <t>2026-03-03 20:05:25</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-03-01 20:26:01</t>
+          <t>2026-03-03 20:15:42</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-03-01 20:25:48</t>
+          <t>2026-03-03 20:05:04</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">

</xml_diff>